<commit_message>
Complete USD defaults and expand currency options
</commit_message>
<xml_diff>
--- a/downloads/inventory/dixani-inventory-master-list.xlsx
+++ b/downloads/inventory/dixani-inventory-master-list.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Master" sheetId="1" r:id="R6718ffeca105478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Lists" sheetId="2" r:id="R108a955577ea4a78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R45fda2423d334095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="Rb1aa388cd3d246d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory Master" sheetId="1" r:id="Ra65911625b594119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Lists" sheetId="2" r:id="R6e1699374fcc413e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to Use" sheetId="3" r:id="R613a44249ff24c51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R99427dad394440d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,7 +98,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="68">
+  <x:cellXfs count="70">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -243,6 +243,12 @@
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -254,7 +260,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -265,7 +271,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -276,7 +282,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -287,7 +293,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -297,7 +303,7 @@
         <x:color rgb="FF15803D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -308,7 +314,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -585,7 +591,7 @@
       <x:c r="T2" s="12"/>
       <x:c r="U2" s="12"/>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="16" t="str">
         <x:v>Company / Business</x:v>
       </x:c>
@@ -598,25 +604,27 @@
         <x:v>Last Updated</x:v>
       </x:c>
       <x:c r="F4" t="str"/>
-      <x:c r="G4" s="16" t="str">
+      <x:c r="G4" s="68" t="str">
         <x:v>Default Currency</x:v>
       </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="H4" s="48" t="str">
         <x:v>QAR</x:v>
       </x:c>
-      <x:c r="I4" t="str"/>
-      <x:c r="J4" t="str"/>
-      <x:c r="K4" t="str"/>
-      <x:c r="L4" t="str"/>
-      <x:c r="M4" t="str"/>
-      <x:c r="N4" t="str"/>
-      <x:c r="O4" t="str"/>
-      <x:c r="P4" t="str"/>
-      <x:c r="Q4" t="str"/>
-      <x:c r="R4" t="str"/>
-      <x:c r="S4" t="str"/>
-      <x:c r="T4" t="str"/>
-      <x:c r="U4" t="str"/>
+      <x:c r="I4" s="69" t="str">
+        <x:v>USD</x:v>
+      </x:c>
+      <x:c r="J4" s="69" t="str"/>
+      <x:c r="K4" s="69" t="str"/>
+      <x:c r="L4" s="69" t="str"/>
+      <x:c r="M4" s="69" t="str"/>
+      <x:c r="N4" s="69" t="str"/>
+      <x:c r="O4" s="69" t="str"/>
+      <x:c r="P4" s="69" t="str"/>
+      <x:c r="Q4" s="69" t="str"/>
+      <x:c r="R4" s="69" t="str"/>
+      <x:c r="S4" s="69" t="str"/>
+      <x:c r="T4" s="69" t="str"/>
+      <x:c r="U4" s="69" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="16" t="str">
@@ -3775,9 +3783,6 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="5">
-    <x:dataValidation type="list" sqref="G4">
-      <x:formula1>"QAR,USD,EUR,GBP,AED,SAR,LKR,INR"</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" sqref="G13:G112">
       <x:formula1>"PCS,EA,BOX,CTN,KG,G,L,ML,M,SET,PACK"</x:formula1>
     </x:dataValidation>
@@ -3789,6 +3794,9 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="U13:U112">
       <x:formula1>"Active,Inactive,Discontinued,On Hold"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I4">
+      <x:formula1>"USD,EUR,GBP,CAD,AUD,NZD,CHF,JPY,CNY,HKD,SGD,INR,AED,SAR,QAR,LKR,ZAR,BRL,MXN"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>